<commit_message>
update of Potentiale.xlsx and literatur_Manual.bib caused by adding new models
git-svn-id: https://scm.projects.hlrs.de/authscm/sleyh/svn/ms2@544 a2be33b2-7eaf-4dce-bf61-b02fde6c56c2
</commit_message>
<xml_diff>
--- a/pmFiles/Potentiale.xlsx
+++ b/pmFiles/Potentiale.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
     <workbookView xWindow="270" yWindow="0" windowWidth="10245" windowHeight="11745" firstSheet="1" activeTab="1"/>
@@ -20,7 +20,7 @@
     <author>Autor</author>
   </authors>
   <commentList>
-    <comment ref="I56" authorId="0">
+    <comment ref="I56" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -44,7 +44,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A69" authorId="0">
+    <comment ref="A69" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2958" uniqueCount="888">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3032" uniqueCount="912">
   <si>
     <t>1CLJ.pm</t>
   </si>
@@ -2737,13 +2737,85 @@
   </si>
   <si>
     <t>take care: read paper carefully-&gt; tab. 2 not Z-martix from pm file -&gt; read tab. 3</t>
+  </si>
+  <si>
+    <t>C3H6O.pm</t>
+  </si>
+  <si>
+    <t>67-64-1</t>
+  </si>
+  <si>
+    <t>Acetone</t>
+  </si>
+  <si>
+    <t>\parencite{Windmann2013}</t>
+  </si>
+  <si>
+    <t>\parencite{Vrabec2006}</t>
+  </si>
+  <si>
+    <t>Ar_tr_sh.pm</t>
+  </si>
+  <si>
+    <t>CH4_tr_sh.pm</t>
+  </si>
+  <si>
+    <t>Kr_tr_sh.pm</t>
+  </si>
+  <si>
+    <t>Xe_tr_sh.pm</t>
+  </si>
+  <si>
+    <t>1 L.J. Center truncated and shifted</t>
+  </si>
+  <si>
+    <t>Ar_I.pm</t>
+  </si>
+  <si>
+    <t>Ar_II.pm</t>
+  </si>
+  <si>
+    <t>Ar\_I.pm</t>
+  </si>
+  <si>
+    <t>Ar\_II.pm</t>
+  </si>
+  <si>
+    <t>CH4_I.pm</t>
+  </si>
+  <si>
+    <t>CH4\_.pm</t>
+  </si>
+  <si>
+    <t>CH4\_II.pm</t>
+  </si>
+  <si>
+    <t>CH4_II.pm</t>
+  </si>
+  <si>
+    <t>Kr_I.pm</t>
+  </si>
+  <si>
+    <t>Kr_II.pm</t>
+  </si>
+  <si>
+    <t>Xe_I.pm</t>
+  </si>
+  <si>
+    <t>Xe\_I.pm</t>
+  </si>
+  <si>
+    <t>Xe_II.pm</t>
+  </si>
+  <si>
+    <t>Xe\_II.pm</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2792,8 +2864,20 @@
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2818,6 +2902,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -2831,7 +2921,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2854,12 +2944,18 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -3261,21 +3357,20 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:P204" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
-  <autoFilter ref="A1:P204">
-    <filterColumn colId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:P208" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
+  <autoFilter ref="A1:P208">
+    <filterColumn colId="6">
       <filters>
-        <filter val="\parencite{Munoz2015}"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="15">
-      <filters>
-        <filter val="pm\ok"/>
+        <filter val="Acetone"/>
+        <filter val="Acetonitrile"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -3305,9 +3400,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Larissa">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Larissa">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3345,9 +3440,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Larissa">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -3382,7 +3477,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -3417,7 +3512,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Larissa">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3635,13 +3730,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P324"/>
+  <dimension ref="A1:P329"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="21.85546875" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="21" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" customWidth="1"/>
     <col min="3" max="3" width="11.140625" customWidth="1"/>
-    <col min="4" max="4" width="8.7109375" customWidth="1"/>
+    <col min="4" max="4" width="9.28515625" customWidth="1"/>
     <col min="5" max="5" width="5" customWidth="1"/>
     <col min="6" max="6" width="15.5703125" customWidth="1"/>
     <col min="7" max="7" width="34.42578125" customWidth="1"/>
@@ -3652,7 +3747,7 @@
     <col min="12" max="12" width="12.5703125" customWidth="1"/>
     <col min="13" max="13" width="36" customWidth="1"/>
     <col min="14" max="14" width="36.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="52" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="52" customWidth="1"/>
     <col min="16" max="16" width="26.85546875" customWidth="1"/>
     <col min="17" max="16384" width="9.140625" style="3"/>
   </cols>
@@ -3850,17 +3945,17 @@
       </c>
     </row>
     <row r="5" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>1</v>
+      <c r="B5" s="21" t="s">
+        <v>898</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>900</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>692</v>
@@ -5159,7 +5254,7 @@
         <v>821</v>
       </c>
     </row>
-    <row r="33" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>343</v>
       </c>
@@ -5205,7 +5300,7 @@
         <v>821</v>
       </c>
     </row>
-    <row r="34" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>328</v>
       </c>
@@ -5253,7 +5348,7 @@
         <v>821</v>
       </c>
     </row>
-    <row r="35" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>327</v>
       </c>
@@ -6375,7 +6470,7 @@
         <v>821</v>
       </c>
     </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>333</v>
       </c>
@@ -6565,7 +6660,7 @@
         <v>821</v>
       </c>
     </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>334</v>
       </c>
@@ -6613,7 +6708,7 @@
         <v>821</v>
       </c>
     </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>335</v>
       </c>
@@ -6661,7 +6756,7 @@
         <v>821</v>
       </c>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>336</v>
       </c>
@@ -6757,7 +6852,7 @@
         <v>821</v>
       </c>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>337</v>
       </c>
@@ -6805,7 +6900,7 @@
         <v>821</v>
       </c>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>338</v>
       </c>
@@ -8454,17 +8549,17 @@
       </c>
     </row>
     <row r="103" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A103" s="1" t="s">
+      <c r="A103" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="B103" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C103" s="1" t="s">
-        <v>38</v>
+      <c r="B103" s="21" t="s">
+        <v>902</v>
+      </c>
+      <c r="C103" s="21" t="s">
+        <v>903</v>
       </c>
       <c r="D103" s="1" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="E103" s="1" t="s">
         <v>692</v>
@@ -9672,17 +9767,17 @@
       </c>
     </row>
     <row r="129" spans="1:16" s="9" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A129" s="1" t="s">
+      <c r="A129" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="B129" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="C129" s="1" t="s">
-        <v>69</v>
+      <c r="B129" s="21" t="s">
+        <v>906</v>
+      </c>
+      <c r="C129" s="21" t="s">
+        <v>906</v>
       </c>
       <c r="D129" s="1" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="E129" s="1" t="s">
         <v>692</v>
@@ -11114,7 +11209,7 @@
         <v>1</v>
       </c>
       <c r="D160" s="1" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="E160" s="1" t="s">
         <v>692</v>
@@ -11160,7 +11255,7 @@
         <v>70</v>
       </c>
       <c r="D161" s="1" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="E161" s="1" t="s">
         <v>824</v>
@@ -11206,7 +11301,7 @@
         <v>72</v>
       </c>
       <c r="D162" s="1" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="E162" s="1" t="s">
         <v>824</v>
@@ -11254,7 +11349,7 @@
         <v>111</v>
       </c>
       <c r="D163" s="1" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="E163" s="1" t="s">
         <v>824</v>
@@ -12944,17 +13039,17 @@
       </c>
     </row>
     <row r="200" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A200" s="1" t="s">
+      <c r="A200" s="21" t="s">
         <v>110</v>
       </c>
-      <c r="B200" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="C200" s="1" t="s">
-        <v>110</v>
+      <c r="B200" s="21" t="s">
+        <v>908</v>
+      </c>
+      <c r="C200" s="21" t="s">
+        <v>909</v>
       </c>
       <c r="D200" s="1" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="E200" s="1" t="s">
         <v>692</v>
@@ -13125,157 +13220,283 @@
         <v>820</v>
       </c>
     </row>
-    <row r="204" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A204" s="1"/>
-      <c r="B204" s="1"/>
-      <c r="C204" s="1"/>
-      <c r="D204" s="1"/>
-      <c r="E204" s="1"/>
-      <c r="F204" s="1"/>
-      <c r="G204" s="1"/>
-      <c r="H204" s="1"/>
-      <c r="I204" s="1"/>
-      <c r="J204" s="1"/>
+    <row r="204" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A204" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="B204" s="1" t="s">
+        <v>888</v>
+      </c>
+      <c r="C204" s="1" t="s">
+        <v>888</v>
+      </c>
+      <c r="D204" s="1" t="s">
+        <v>832</v>
+      </c>
+      <c r="E204" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="F204" t="s">
+        <v>889</v>
+      </c>
+      <c r="G204" s="8" t="s">
+        <v>890</v>
+      </c>
+      <c r="H204" s="8" t="s">
+        <v>890</v>
+      </c>
+      <c r="I204" s="1" t="s">
+        <v>891</v>
+      </c>
+      <c r="J204" s="1" t="s">
+        <v>650</v>
+      </c>
       <c r="K204" s="1"/>
-      <c r="L204" s="1"/>
-      <c r="M204" s="1"/>
-      <c r="N204" s="1"/>
-      <c r="O204" s="1"/>
-      <c r="P204" s="1"/>
-    </row>
-    <row r="205" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="I205" s="3"/>
-      <c r="J205" s="3"/>
-      <c r="K205" s="3"/>
-      <c r="L205" s="3"/>
-      <c r="M205" s="3"/>
-      <c r="N205" s="3"/>
-      <c r="O205" s="3"/>
-      <c r="P205" s="3"/>
-    </row>
-    <row r="206" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="I206" s="3"/>
-      <c r="J206" s="3"/>
-      <c r="K206" s="3"/>
-      <c r="L206" s="3"/>
-      <c r="M206" s="3"/>
-      <c r="N206" s="3"/>
-      <c r="O206" s="3"/>
-      <c r="P206" s="3"/>
-    </row>
-    <row r="207" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A207" s="3" t="s">
-        <v>847</v>
-      </c>
-      <c r="B207" s="3" t="s">
-        <v>848</v>
-      </c>
-      <c r="C207" s="3" t="s">
-        <v>849</v>
-      </c>
-      <c r="D207" s="3" t="s">
-        <v>859</v>
-      </c>
-      <c r="E207" s="3" t="s">
-        <v>850</v>
-      </c>
-      <c r="F207" s="3"/>
-      <c r="G207" s="7" t="s">
-        <v>851</v>
-      </c>
-      <c r="H207" s="7" t="s">
-        <v>852</v>
-      </c>
-      <c r="I207" s="7" t="s">
-        <v>853</v>
-      </c>
-      <c r="J207" s="3"/>
-      <c r="K207" s="3"/>
-      <c r="L207" s="3" t="s">
-        <v>854</v>
-      </c>
-      <c r="M207" s="3"/>
-      <c r="N207" s="3" t="s">
-        <v>855</v>
-      </c>
-      <c r="O207" s="3"/>
-      <c r="P207" s="3"/>
-    </row>
-    <row r="208" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A208" s="3" t="s">
-        <v>589</v>
-      </c>
-      <c r="B208" s="16" t="s">
-        <v>563</v>
-      </c>
-      <c r="C208" s="16"/>
-      <c r="D208" s="16"/>
-      <c r="E208" s="16"/>
-      <c r="F208" s="3"/>
-      <c r="G208" s="17" t="s">
-        <v>564</v>
-      </c>
-      <c r="H208" s="17"/>
-      <c r="I208" s="3"/>
-      <c r="J208" s="3"/>
-      <c r="K208" s="3"/>
-      <c r="L208" s="3"/>
-      <c r="M208" s="3"/>
-      <c r="N208" s="3"/>
-      <c r="O208" s="3"/>
-      <c r="P208" s="3"/>
+      <c r="L204" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="M204" s="1" t="s">
+        <v>861</v>
+      </c>
+      <c r="N204" s="1" t="s">
+        <v>708</v>
+      </c>
+      <c r="O204" s="1" t="s">
+        <v>824</v>
+      </c>
+      <c r="P204" s="1" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="205" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A205" s="21" t="s">
+        <v>893</v>
+      </c>
+      <c r="B205" s="21" t="s">
+        <v>899</v>
+      </c>
+      <c r="C205" s="21" t="s">
+        <v>901</v>
+      </c>
+      <c r="D205" s="1" t="s">
+        <v>836</v>
+      </c>
+      <c r="E205" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="F205" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="G205" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="H205" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="I205" s="1" t="s">
+        <v>892</v>
+      </c>
+      <c r="J205" s="1" t="s">
+        <v>897</v>
+      </c>
+      <c r="K205" s="1"/>
+      <c r="L205" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="M205" s="1" t="s">
+        <v>861</v>
+      </c>
+      <c r="N205" s="1" t="s">
+        <v>708</v>
+      </c>
+      <c r="O205" s="1" t="s">
+        <v>824</v>
+      </c>
+      <c r="P205" s="1" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="206" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A206" s="21" t="s">
+        <v>894</v>
+      </c>
+      <c r="B206" s="21" t="s">
+        <v>905</v>
+      </c>
+      <c r="C206" s="21" t="s">
+        <v>904</v>
+      </c>
+      <c r="D206" s="1" t="s">
+        <v>836</v>
+      </c>
+      <c r="E206" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="F206" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="G206" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="H206" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="I206" s="1" t="s">
+        <v>892</v>
+      </c>
+      <c r="J206" s="1" t="s">
+        <v>897</v>
+      </c>
+      <c r="K206" s="1"/>
+      <c r="L206" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="M206" s="1" t="s">
+        <v>861</v>
+      </c>
+      <c r="N206" s="1" t="s">
+        <v>708</v>
+      </c>
+      <c r="O206" s="1" t="s">
+        <v>824</v>
+      </c>
+      <c r="P206" s="1" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="207" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A207" s="21" t="s">
+        <v>895</v>
+      </c>
+      <c r="B207" s="21" t="s">
+        <v>907</v>
+      </c>
+      <c r="C207" s="21" t="s">
+        <v>907</v>
+      </c>
+      <c r="D207" s="1" t="s">
+        <v>836</v>
+      </c>
+      <c r="E207" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="F207" t="s">
+        <v>183</v>
+      </c>
+      <c r="G207" s="8" t="s">
+        <v>429</v>
+      </c>
+      <c r="H207" s="8" t="s">
+        <v>429</v>
+      </c>
+      <c r="I207" s="1" t="s">
+        <v>892</v>
+      </c>
+      <c r="J207" s="1" t="s">
+        <v>897</v>
+      </c>
+      <c r="K207" s="1"/>
+      <c r="L207" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="M207" s="1" t="s">
+        <v>861</v>
+      </c>
+      <c r="N207" s="1" t="s">
+        <v>708</v>
+      </c>
+      <c r="O207" s="1" t="s">
+        <v>824</v>
+      </c>
+      <c r="P207" s="1" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="208" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A208" s="21" t="s">
+        <v>896</v>
+      </c>
+      <c r="B208" s="21" t="s">
+        <v>910</v>
+      </c>
+      <c r="C208" s="21" t="s">
+        <v>911</v>
+      </c>
+      <c r="D208" s="1" t="s">
+        <v>836</v>
+      </c>
+      <c r="E208" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="F208" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="G208" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="H208" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="I208" s="1" t="s">
+        <v>892</v>
+      </c>
+      <c r="J208" s="1" t="s">
+        <v>897</v>
+      </c>
+      <c r="K208" s="1"/>
+      <c r="L208" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="M208" s="1" t="s">
+        <v>861</v>
+      </c>
+      <c r="N208" s="1" t="s">
+        <v>708</v>
+      </c>
+      <c r="O208" s="1" t="s">
+        <v>824</v>
+      </c>
+      <c r="P208" s="1" t="s">
+        <v>821</v>
+      </c>
     </row>
     <row r="209" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A209" s="3"/>
-      <c r="B209" s="3"/>
-      <c r="C209" s="3"/>
-      <c r="D209" s="3"/>
-      <c r="E209" s="3"/>
-      <c r="F209" s="3"/>
-      <c r="G209" s="3"/>
-      <c r="H209" s="3"/>
-      <c r="I209" s="3"/>
-      <c r="J209" s="3"/>
-      <c r="K209" s="3"/>
-      <c r="L209" s="3"/>
-      <c r="M209" s="3"/>
-      <c r="N209" s="3"/>
-      <c r="O209" s="3"/>
-      <c r="P209" s="3"/>
+      <c r="A209" s="1"/>
+      <c r="B209" s="1"/>
+      <c r="C209" s="1"/>
+      <c r="D209" s="1"/>
+      <c r="E209" s="1"/>
+      <c r="F209" s="1"/>
+      <c r="G209" s="4"/>
+      <c r="H209" s="4"/>
+      <c r="I209" s="1"/>
+      <c r="J209" s="1"/>
+      <c r="K209" s="1"/>
+      <c r="L209" s="1"/>
+      <c r="M209" s="1"/>
+      <c r="N209" s="1"/>
+      <c r="O209" s="1"/>
+      <c r="P209" s="1"/>
     </row>
     <row r="210" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A210" s="3"/>
-      <c r="B210" s="3"/>
-      <c r="C210" s="3"/>
-      <c r="D210" s="3"/>
-      <c r="E210" s="3"/>
-      <c r="F210" s="3"/>
-      <c r="G210" s="3"/>
-      <c r="H210" s="3"/>
-      <c r="I210" s="3"/>
-      <c r="J210" s="3"/>
-      <c r="K210" s="3"/>
-      <c r="L210" s="3"/>
-      <c r="M210" s="3"/>
-      <c r="N210" s="3"/>
-      <c r="O210" s="3"/>
-      <c r="P210" s="3"/>
+      <c r="A210" s="16"/>
+      <c r="B210" s="16"/>
+      <c r="C210" s="16"/>
+      <c r="D210" s="16"/>
+      <c r="E210" s="1"/>
+      <c r="F210" s="16"/>
+      <c r="G210" s="16"/>
+      <c r="H210" s="16"/>
+      <c r="I210" s="1"/>
+      <c r="J210" s="16"/>
+      <c r="K210" s="16"/>
+      <c r="L210" s="1"/>
+      <c r="M210" s="1"/>
+      <c r="N210" s="1"/>
+      <c r="O210" s="1"/>
+      <c r="P210" s="1"/>
     </row>
     <row r="211" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A211" s="3" t="s">
-        <v>670</v>
-      </c>
-      <c r="B211" s="3">
-        <v>0</v>
-      </c>
-      <c r="C211" s="3" t="s">
-        <v>845</v>
-      </c>
-      <c r="D211" s="3"/>
-      <c r="E211" s="3"/>
-      <c r="F211" s="3"/>
-      <c r="G211" s="3"/>
-      <c r="H211" s="3"/>
       <c r="I211" s="3"/>
       <c r="J211" s="3"/>
       <c r="K211" s="3"/>
@@ -13287,39 +13508,57 @@
     </row>
     <row r="212" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A212" s="3" t="s">
-        <v>667</v>
-      </c>
-      <c r="B212" s="3"/>
-      <c r="C212" s="3"/>
-      <c r="D212" s="3"/>
-      <c r="E212" s="3"/>
+        <v>847</v>
+      </c>
+      <c r="B212" s="3" t="s">
+        <v>848</v>
+      </c>
+      <c r="C212" s="3" t="s">
+        <v>849</v>
+      </c>
+      <c r="D212" s="3" t="s">
+        <v>859</v>
+      </c>
+      <c r="E212" s="3" t="s">
+        <v>850</v>
+      </c>
       <c r="F212" s="3"/>
-      <c r="G212" s="3"/>
-      <c r="H212" s="3"/>
-      <c r="I212" s="3"/>
+      <c r="G212" s="7" t="s">
+        <v>851</v>
+      </c>
+      <c r="H212" s="7" t="s">
+        <v>852</v>
+      </c>
+      <c r="I212" s="7" t="s">
+        <v>853</v>
+      </c>
       <c r="J212" s="3"/>
       <c r="K212" s="3"/>
-      <c r="L212" s="3"/>
+      <c r="L212" s="3" t="s">
+        <v>854</v>
+      </c>
       <c r="M212" s="3"/>
-      <c r="N212" s="3"/>
+      <c r="N212" s="3" t="s">
+        <v>855</v>
+      </c>
       <c r="O212" s="3"/>
       <c r="P212" s="3"/>
     </row>
     <row r="213" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A213" s="3" t="s">
-        <v>667</v>
-      </c>
-      <c r="B213" s="3">
-        <v>1</v>
-      </c>
-      <c r="C213" s="3" t="s">
-        <v>843</v>
-      </c>
-      <c r="D213" s="3"/>
-      <c r="E213" s="3"/>
+        <v>589</v>
+      </c>
+      <c r="B213" s="18" t="s">
+        <v>563</v>
+      </c>
+      <c r="C213" s="18"/>
+      <c r="D213" s="18"/>
+      <c r="E213" s="18"/>
       <c r="F213" s="3"/>
-      <c r="G213" s="3"/>
-      <c r="H213" s="3"/>
+      <c r="G213" s="19" t="s">
+        <v>564</v>
+      </c>
+      <c r="H213" s="19"/>
       <c r="I213" s="3"/>
       <c r="J213" s="3"/>
       <c r="K213" s="3"/>
@@ -13330,14 +13569,10 @@
       <c r="P213" s="3"/>
     </row>
     <row r="214" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A214" s="3" t="s">
-        <v>667</v>
-      </c>
+      <c r="A214" s="3"/>
       <c r="B214" s="3"/>
-      <c r="C214" s="1" t="s">
-        <v>821</v>
-      </c>
-      <c r="D214" s="1"/>
+      <c r="C214" s="3"/>
+      <c r="D214" s="3"/>
       <c r="E214" s="3"/>
       <c r="F214" s="3"/>
       <c r="G214" s="3"/>
@@ -13352,35 +13587,33 @@
       <c r="P214" s="3"/>
     </row>
     <row r="215" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A215" s="3" t="s">
-        <v>667</v>
-      </c>
+      <c r="A215" s="3"/>
       <c r="B215" s="3"/>
-      <c r="C215" s="1"/>
-      <c r="D215" s="1"/>
+      <c r="C215" s="3"/>
+      <c r="D215" s="3"/>
       <c r="E215" s="3"/>
       <c r="F215" s="3"/>
-      <c r="G215" s="1"/>
-      <c r="H215" s="1"/>
-      <c r="I215" s="1"/>
-      <c r="J215" s="1"/>
-      <c r="K215" s="1"/>
-      <c r="L215" s="1"/>
-      <c r="M215" s="1"/>
-      <c r="N215" s="1" t="s">
-        <v>730</v>
-      </c>
-      <c r="O215" s="1" t="s">
-        <v>660</v>
-      </c>
-      <c r="P215" s="1"/>
+      <c r="G215" s="3"/>
+      <c r="H215" s="3"/>
+      <c r="I215" s="3"/>
+      <c r="J215" s="3"/>
+      <c r="K215" s="3"/>
+      <c r="L215" s="3"/>
+      <c r="M215" s="3"/>
+      <c r="N215" s="3"/>
+      <c r="O215" s="3"/>
+      <c r="P215" s="3"/>
     </row>
     <row r="216" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A216" s="3" t="s">
-        <v>667</v>
-      </c>
-      <c r="B216" s="3"/>
-      <c r="C216" s="3"/>
+        <v>670</v>
+      </c>
+      <c r="B216" s="3">
+        <v>0</v>
+      </c>
+      <c r="C216" s="3" t="s">
+        <v>845</v>
+      </c>
       <c r="D216" s="3"/>
       <c r="E216" s="3"/>
       <c r="F216" s="3"/>
@@ -13399,12 +13632,8 @@
       <c r="A217" s="3" t="s">
         <v>667</v>
       </c>
-      <c r="B217" s="3">
-        <v>2</v>
-      </c>
-      <c r="C217" s="3" t="s">
-        <v>842</v>
-      </c>
+      <c r="B217" s="3"/>
+      <c r="C217" s="3"/>
       <c r="D217" s="3"/>
       <c r="E217" s="3"/>
       <c r="F217" s="3"/>
@@ -13423,9 +13652,11 @@
       <c r="A218" s="3" t="s">
         <v>667</v>
       </c>
-      <c r="B218" s="3"/>
+      <c r="B218" s="3">
+        <v>1</v>
+      </c>
       <c r="C218" s="3" t="s">
-        <v>668</v>
+        <v>843</v>
       </c>
       <c r="D218" s="3"/>
       <c r="E218" s="3"/>
@@ -13446,8 +13677,10 @@
         <v>667</v>
       </c>
       <c r="B219" s="3"/>
-      <c r="C219" s="3"/>
-      <c r="D219" s="3"/>
+      <c r="C219" s="1" t="s">
+        <v>821</v>
+      </c>
+      <c r="D219" s="1"/>
       <c r="E219" s="3"/>
       <c r="F219" s="3"/>
       <c r="G219" s="3"/>
@@ -13465,34 +13698,30 @@
       <c r="A220" s="3" t="s">
         <v>667</v>
       </c>
-      <c r="B220" s="3">
-        <v>3</v>
-      </c>
-      <c r="C220" s="3" t="s">
-        <v>672</v>
-      </c>
-      <c r="D220" s="3"/>
+      <c r="B220" s="3"/>
+      <c r="C220" s="1"/>
+      <c r="D220" s="1"/>
       <c r="E220" s="3"/>
       <c r="F220" s="3"/>
-      <c r="G220" s="3"/>
-      <c r="H220" s="3"/>
-      <c r="I220" s="3"/>
-      <c r="J220" s="3"/>
-      <c r="K220" s="3"/>
-      <c r="L220" s="3"/>
-      <c r="M220" s="3"/>
-      <c r="N220" s="3"/>
-      <c r="O220" s="3"/>
-      <c r="P220" s="3"/>
+      <c r="G220" s="1"/>
+      <c r="H220" s="1"/>
+      <c r="I220" s="1"/>
+      <c r="J220" s="1"/>
+      <c r="K220" s="1"/>
+      <c r="L220" s="1"/>
+      <c r="M220" s="1"/>
+      <c r="N220" s="1" t="s">
+        <v>730</v>
+      </c>
+      <c r="O220" s="1"/>
+      <c r="P220" s="1"/>
     </row>
     <row r="221" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A221" s="3" t="s">
         <v>667</v>
       </c>
       <c r="B221" s="3"/>
-      <c r="C221" s="3" t="s">
-        <v>673</v>
-      </c>
+      <c r="C221" s="3"/>
       <c r="D221" s="3"/>
       <c r="E221" s="3"/>
       <c r="F221" s="3"/>
@@ -13511,9 +13740,11 @@
       <c r="A222" s="3" t="s">
         <v>667</v>
       </c>
-      <c r="B222" s="3"/>
+      <c r="B222" s="3">
+        <v>2</v>
+      </c>
       <c r="C222" s="3" t="s">
-        <v>674</v>
+        <v>842</v>
       </c>
       <c r="D222" s="3"/>
       <c r="E222" s="3"/>
@@ -13534,13 +13765,15 @@
         <v>667</v>
       </c>
       <c r="B223" s="3"/>
-      <c r="C223" s="3"/>
+      <c r="C223" s="3" t="s">
+        <v>668</v>
+      </c>
       <c r="D223" s="3"/>
       <c r="E223" s="3"/>
       <c r="F223" s="3"/>
       <c r="G223" s="3"/>
       <c r="H223" s="3"/>
-      <c r="I223" s="3"/>
+      <c r="I223" s="17"/>
       <c r="J223" s="3"/>
       <c r="K223" s="3"/>
       <c r="L223" s="3"/>
@@ -13553,12 +13786,8 @@
       <c r="A224" s="3" t="s">
         <v>667</v>
       </c>
-      <c r="B224" s="3">
-        <v>4</v>
-      </c>
-      <c r="C224" s="3" t="s">
-        <v>669</v>
-      </c>
+      <c r="B224" s="3"/>
+      <c r="C224" s="3"/>
       <c r="D224" s="3"/>
       <c r="E224" s="3"/>
       <c r="F224" s="3"/>
@@ -13577,8 +13806,12 @@
       <c r="A225" s="3" t="s">
         <v>667</v>
       </c>
-      <c r="B225" s="3"/>
-      <c r="C225" s="3"/>
+      <c r="B225" s="3">
+        <v>3</v>
+      </c>
+      <c r="C225" s="3" t="s">
+        <v>672</v>
+      </c>
       <c r="D225" s="3"/>
       <c r="E225" s="3"/>
       <c r="F225" s="3"/>
@@ -13597,11 +13830,9 @@
       <c r="A226" s="3" t="s">
         <v>667</v>
       </c>
-      <c r="B226" s="3">
-        <v>5</v>
-      </c>
+      <c r="B226" s="3"/>
       <c r="C226" s="3" t="s">
-        <v>765</v>
+        <v>673</v>
       </c>
       <c r="D226" s="3"/>
       <c r="E226" s="3"/>
@@ -13623,7 +13854,7 @@
       </c>
       <c r="B227" s="3"/>
       <c r="C227" s="3" t="s">
-        <v>844</v>
+        <v>674</v>
       </c>
       <c r="D227" s="3"/>
       <c r="E227" s="3"/>
@@ -13660,12 +13891,14 @@
       <c r="P228" s="3"/>
     </row>
     <row r="229" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A229" s="3"/>
+      <c r="A229" s="3" t="s">
+        <v>667</v>
+      </c>
       <c r="B229" s="3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C229" s="3" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="D229" s="3"/>
       <c r="E229" s="3"/>
@@ -13682,7 +13915,9 @@
       <c r="P229" s="3"/>
     </row>
     <row r="230" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A230" s="3"/>
+      <c r="A230" s="3" t="s">
+        <v>667</v>
+      </c>
       <c r="B230" s="3"/>
       <c r="C230" s="3"/>
       <c r="D230" s="3"/>
@@ -13700,9 +13935,15 @@
       <c r="P230" s="3"/>
     </row>
     <row r="231" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A231" s="3"/>
-      <c r="B231" s="3"/>
-      <c r="C231" s="3"/>
+      <c r="A231" s="3" t="s">
+        <v>667</v>
+      </c>
+      <c r="B231" s="3">
+        <v>5</v>
+      </c>
+      <c r="C231" s="3" t="s">
+        <v>765</v>
+      </c>
       <c r="D231" s="3"/>
       <c r="E231" s="3"/>
       <c r="F231" s="3"/>
@@ -13718,9 +13959,13 @@
       <c r="P231" s="3"/>
     </row>
     <row r="232" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A232" s="3"/>
+      <c r="A232" s="3" t="s">
+        <v>667</v>
+      </c>
       <c r="B232" s="3"/>
-      <c r="C232" s="3"/>
+      <c r="C232" s="3" t="s">
+        <v>844</v>
+      </c>
       <c r="D232" s="3"/>
       <c r="E232" s="3"/>
       <c r="F232" s="3"/>
@@ -13736,7 +13981,9 @@
       <c r="P232" s="3"/>
     </row>
     <row r="233" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A233" s="3"/>
+      <c r="A233" s="3" t="s">
+        <v>667</v>
+      </c>
       <c r="B233" s="3"/>
       <c r="C233" s="3"/>
       <c r="D233" s="3"/>
@@ -13755,8 +14002,12 @@
     </row>
     <row r="234" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A234" s="3"/>
-      <c r="B234" s="3"/>
-      <c r="C234" s="3"/>
+      <c r="B234" s="3">
+        <v>6</v>
+      </c>
+      <c r="C234" s="3" t="s">
+        <v>671</v>
+      </c>
       <c r="D234" s="3"/>
       <c r="E234" s="3"/>
       <c r="F234" s="3"/>
@@ -15374,19 +15625,109 @@
       <c r="P323" s="3"/>
     </row>
     <row r="324" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A324" s="3"/>
       <c r="B324" s="3"/>
       <c r="C324" s="3"/>
       <c r="D324" s="3"/>
       <c r="E324" s="3"/>
       <c r="F324" s="3"/>
+      <c r="G324" s="3"/>
+      <c r="H324" s="3"/>
+      <c r="I324" s="3"/>
+      <c r="J324" s="3"/>
+      <c r="K324" s="3"/>
+      <c r="L324" s="3"/>
+      <c r="M324" s="3"/>
+      <c r="N324" s="3"/>
+      <c r="O324" s="3"/>
+      <c r="P324" s="3"/>
+    </row>
+    <row r="325" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A325" s="3"/>
+      <c r="B325" s="3"/>
+      <c r="C325" s="3"/>
+      <c r="D325" s="3"/>
+      <c r="E325" s="3"/>
+      <c r="F325" s="3"/>
+      <c r="G325" s="3"/>
+      <c r="H325" s="3"/>
+      <c r="I325" s="3"/>
+      <c r="J325" s="3"/>
+      <c r="K325" s="3"/>
+      <c r="L325" s="3"/>
+      <c r="M325" s="3"/>
+      <c r="N325" s="3"/>
+      <c r="O325" s="3"/>
+      <c r="P325" s="3"/>
+    </row>
+    <row r="326" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A326" s="3"/>
+      <c r="B326" s="3"/>
+      <c r="C326" s="3"/>
+      <c r="D326" s="3"/>
+      <c r="E326" s="3"/>
+      <c r="F326" s="3"/>
+      <c r="G326" s="3"/>
+      <c r="H326" s="3"/>
+      <c r="I326" s="3"/>
+      <c r="J326" s="3"/>
+      <c r="K326" s="3"/>
+      <c r="L326" s="3"/>
+      <c r="M326" s="3"/>
+      <c r="N326" s="3"/>
+      <c r="O326" s="3"/>
+      <c r="P326" s="3"/>
+    </row>
+    <row r="327" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A327" s="3"/>
+      <c r="B327" s="3"/>
+      <c r="C327" s="3"/>
+      <c r="D327" s="3"/>
+      <c r="E327" s="3"/>
+      <c r="F327" s="3"/>
+      <c r="G327" s="3"/>
+      <c r="H327" s="3"/>
+      <c r="I327" s="3"/>
+      <c r="J327" s="3"/>
+      <c r="K327" s="3"/>
+      <c r="L327" s="3"/>
+      <c r="M327" s="3"/>
+      <c r="N327" s="3"/>
+      <c r="O327" s="3"/>
+      <c r="P327" s="3"/>
+    </row>
+    <row r="328" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A328" s="3"/>
+      <c r="B328" s="3"/>
+      <c r="C328" s="3"/>
+      <c r="D328" s="3"/>
+      <c r="E328" s="3"/>
+      <c r="F328" s="3"/>
+      <c r="G328" s="3"/>
+      <c r="H328" s="3"/>
+      <c r="I328" s="3"/>
+      <c r="J328" s="3"/>
+      <c r="K328" s="3"/>
+      <c r="L328" s="3"/>
+      <c r="M328" s="3"/>
+      <c r="N328" s="3"/>
+      <c r="O328" s="3"/>
+      <c r="P328" s="3"/>
+    </row>
+    <row r="329" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B329" s="3"/>
+      <c r="C329" s="3"/>
+      <c r="D329" s="3"/>
+      <c r="E329" s="3"/>
+      <c r="F329" s="3"/>
     </row>
   </sheetData>
   <sortState ref="A2:A43">
     <sortCondition ref="A1"/>
   </sortState>
   <mergeCells count="2">
-    <mergeCell ref="B208:E208"/>
-    <mergeCell ref="G208:H208"/>
+    <mergeCell ref="B213:E213"/>
+    <mergeCell ref="G213:H213"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
found pub. for modell in diss stoll
git-svn-id: https://scm.projects.hlrs.de/authscm/sleyh/svn/ms2@550 a2be33b2-7eaf-4dce-bf61-b02fde6c56c2
</commit_message>
<xml_diff>
--- a/pmFiles/Potentiale.xlsx
+++ b/pmFiles/Potentiale.xlsx
@@ -3369,7 +3369,7 @@
   <autoFilter ref="A1:P208">
     <filterColumn colId="8">
       <filters>
-        <filter val="\parencite{Deublein2012_A}"/>
+        <filter val="\parencite{Stoll2004}"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -4319,7 +4319,7 @@
         <v>867</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>285</v>
       </c>
@@ -4365,7 +4365,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>286</v>
       </c>
@@ -4551,7 +4551,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="18" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>5</v>
       </c>
@@ -4643,7 +4643,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="20" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>6</v>
       </c>
@@ -5121,7 +5121,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="30" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>7</v>
       </c>
@@ -5259,7 +5259,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="33" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>269</v>
       </c>
@@ -5285,7 +5285,7 @@
         <v>503</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>267</v>
+        <v>115</v>
       </c>
       <c r="J33" s="1" t="s">
         <v>634</v>
@@ -6329,7 +6329,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="56" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>10</v>
       </c>
@@ -7753,7 +7753,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>288</v>
       </c>
@@ -9111,7 +9111,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="115" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
         <v>41</v>
       </c>
@@ -9529,7 +9529,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="124" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
         <v>55</v>
       </c>
@@ -10097,7 +10097,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="136" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136" s="1" t="s">
         <v>294</v>
       </c>
@@ -10143,7 +10143,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="137" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A137" s="1" t="s">
         <v>75</v>
       </c>
@@ -10283,7 +10283,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="140" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A140" s="1" t="s">
         <v>79</v>
       </c>
@@ -11621,7 +11621,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="169" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A169" s="1" t="s">
         <v>456</v>
       </c>
@@ -11669,7 +11669,7 @@
         <v>885</v>
       </c>
     </row>
-    <row r="170" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A170" s="1" t="s">
         <v>457</v>
       </c>
@@ -12991,7 +12991,7 @@
         <v>819</v>
       </c>
     </row>
-    <row r="199" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A199" s="1" t="s">
         <v>458</v>
       </c>
@@ -13039,7 +13039,7 @@
         <v>885</v>
       </c>
     </row>
-    <row r="200" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A200" s="1" t="s">
         <v>459</v>
       </c>
@@ -13229,7 +13229,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="204" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A204" s="1" t="s">
         <v>297</v>
       </c>

</xml_diff>

<commit_message>
error spotted in database (just corrected in database)
git-svn-id: https://scm.projects.hlrs.de/authscm/sleyh/svn/ms2@552 a2be33b2-7eaf-4dce-bf61-b02fde6c56c2
</commit_message>
<xml_diff>
--- a/pmFiles/Potentiale.xlsx
+++ b/pmFiles/Potentiale.xlsx
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3032" uniqueCount="912">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3033" uniqueCount="913">
   <si>
     <t>1CLJ.pm</t>
   </si>
@@ -2809,6 +2809,9 @@
   </si>
   <si>
     <t>Speicherort (alt)</t>
+  </si>
+  <si>
+    <t>corrected (just in Database)</t>
   </si>
 </sst>
 </file>
@@ -3367,9 +3370,9 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:P208" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
   <autoFilter ref="A1:P208">
-    <filterColumn colId="8">
+    <filterColumn colId="1">
       <filters>
-        <filter val="\parencite{Stoll2004}"/>
+        <filter val="CH5N.pm"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -4551,7 +4554,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>5</v>
       </c>
@@ -4643,7 +4646,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>6</v>
       </c>
@@ -5121,7 +5124,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>7</v>
       </c>
@@ -5259,7 +5262,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>269</v>
       </c>
@@ -6329,7 +6332,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>10</v>
       </c>
@@ -8586,7 +8589,7 @@
         <v>694</v>
       </c>
       <c r="N103" s="1" t="s">
-        <v>704</v>
+        <v>912</v>
       </c>
       <c r="O103" s="1" t="s">
         <v>282</v>
@@ -8923,7 +8926,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="111" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
         <v>74</v>
       </c>
@@ -8956,11 +8959,13 @@
       </c>
       <c r="K111" s="1"/>
       <c r="L111" s="1" t="s">
-        <v>691</v>
-      </c>
-      <c r="M111" s="1"/>
+        <v>138</v>
+      </c>
+      <c r="M111" s="1" t="s">
+        <v>694</v>
+      </c>
       <c r="N111" s="1" t="s">
-        <v>703</v>
+        <v>912</v>
       </c>
       <c r="O111" s="1" t="s">
         <v>314</v>
@@ -9111,7 +9116,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="115" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
         <v>41</v>
       </c>
@@ -9529,7 +9534,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="124" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
         <v>55</v>
       </c>
@@ -10143,7 +10148,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="137" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" s="1" t="s">
         <v>75</v>
       </c>
@@ -10283,7 +10288,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="140" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140" s="1" t="s">
         <v>79</v>
       </c>

</xml_diff>